<commit_message>
Consolidate credit/leverage metrics into the main comparison table
Adds Debt/EBITDA, Net Debt/EBITDA, and Interest Coverage columns by
importing fetch_credit_metrics.compute_credit_metrics() the same way
consolidate.py already imports the other modules — nothing recomputed.

The table now reads as two visually separated sections (shaded section
banner + divider in both xlsx and html): moat metrics and credit/
leverage. Credit-metric flags (ETN/PWR using InterestExpenseNonoperating,
NVT's interest coverage on a net rather than gross interest-expense
basis, PWR/NVT D&A derived from components) are carried through as a
dedicated flags block in both outputs so they aren't lost.

Local commit only, not pushed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/consolidated_comparison.xlsx
+++ b/output/consolidated_comparison.xlsx
@@ -16,17 +16,22 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="166" formatCode="+0.0%;-0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
     </font>
     <font>
       <b val="1"/>
@@ -38,13 +43,34 @@
     <font>
       <color rgb="009C0006"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -65,15 +91,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -452,205 +492,332 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="39" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>MOAT METRICS</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>CREDIT / LEVERAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>FY</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Gross Margin</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Gross Margin Spread vs. Peer Avg</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Operating Margin</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Operating Margin Spread vs. Peer Avg</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>ROIC Spread vs. Peer Avg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Customer Concentration</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>VRT</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>10229900000</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0.363170705480992</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>0.04654200326856489</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>0.1788580533534052</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>0.03294462224040129</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>0.2606698241879197</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>0.1150560400722674</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Not disclosed</t>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Net Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Interest Coverage (EBITDA / Interest)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2025</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>27448000000</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0.3758743806470417</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0.05924567843461459</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>0.1897770329350044</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>0.04386360182200044</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>0.1472955008045327</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>0.00168171668888048</v>
+      <c r="C3" s="5" t="n">
+        <v>10229900000</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>0.363170705480992</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.04654200326856489</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>0.1788580533534052</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0.03294462224040129</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>0.2606698241879197</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>0.1150560400722674</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>No customer exceeds 10%</t>
-        </is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>1.476780620118786</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>0.6684749567413366</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>24.83507549361208</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2025</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>28479697000</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0.1501097782044521</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>-0.166518924007975</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>0.05658448543184993</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>-0.08932894568115399</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>0.08162941364077377</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>-0.06398437047487847</v>
+      <c r="C4" s="5" t="n">
+        <v>27448000000</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.3758743806470417</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.05924567843461459</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.1897770329350044</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0.04386360182200044</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.1472955008045327</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0.00168171668888048</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Largest customer: 8%; top 10: 30%</t>
-        </is>
+          <t>No customer exceeds 10%</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>1.69444891391794</v>
+      </c>
+      <c r="L4" s="8" t="n">
+        <v>1.594368463395012</v>
+      </c>
+      <c r="M4" s="8" t="n">
+        <v>25.78838174273859</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>2025</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="5" t="n">
+        <v>28479697000</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.1501097782044521</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>-0.166518924007975</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.05658448543184993</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>-0.08932894568115399</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.08162941364077377</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>-0.06398437047487847</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Largest customer: 8%; top 10: 30%</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>2.49998889700465</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>2.325708351276567</v>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>9.64578400810878</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" s="5" t="n">
         <v>3893100000</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D6" s="6" t="n">
         <v>0.3773599445172228</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.06073124230479565</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F6" s="6" t="n">
         <v>0.1584341527317562</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G6" s="7" t="n">
         <v>0.01252072161875226</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H6" s="6" t="n">
         <v>0.09286039782938273</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I6" s="9" t="n">
         <v>-0.05275338628626951</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Largest customer: 11%</t>
         </is>
       </c>
+      <c r="K6" s="8" t="n">
+        <v>2.040019403347078</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>1.752000970167354</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>10.99466666666667</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Credit / Leverage — flags to hand-check</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>[ETN] InterestExpense tag not reported for FY ended 2025-12-31; used InterestExpenseNonoperating instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>[PWR] No combined DepreciationDepletionAndAmortization tag; D&amp;A derived as Depreciation ($411,538,000) + AmortizationOfIntangibleAssets ($498,795,000) = $910,333,000. Excludes finance-lease right-of-use asset amortization if separately tagged — hand-check against the cash flow statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>[PWR] InterestExpense tag not reported for FY ended 2025-12-31; used InterestExpenseNonoperating instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>[NVT] CashCashEquivalentsRestrictedCashAndRestrictedCashEquivalents used instead of CashAndCashEquivalentsAtCarryingValue — may include a small restricted-cash component — hand-check against the balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>[NVT] No combined DepreciationDepletionAndAmortization tag; D&amp;A derived as Depreciation ($60,700,000) + AmortizationOfIntangibleAssets ($147,100,000) = $207,800,000. Excludes finance-lease right-of-use asset amortization if separately tagged — hand-check against the cash flow statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>[NVT] No gross interest expense tag (InterestExpense / InterestExpenseNonoperating) reported for FY ended 2025-12-31; used |InterestIncomeExpenseNet| = $75,000,000 instead. This is interest expense NET of interest income, not gross interest expense — EBITDA/interest coverage will read stronger than on a gross-expense basis. Hand-check against the filing's interest expense footnote.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A13:M13"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="A12:M12"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="K1:M1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>